<commit_message>
Update template schema, add delivery type, and refresh roadmap visual styling
</commit_message>
<xml_diff>
--- a/templates/roadmap_template.xlsx
+++ b/templates/roadmap_template.xlsx
@@ -11,7 +11,7 @@
     <sheet name="Instructions" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Roadmap'!$A$1:$E$1000</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Roadmap'!$A$1:$F$1000</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -434,14 +434,15 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E1"/>
+  <dimension ref="A1:F1"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="24" customWidth="1" min="1" max="1"/>
     <col width="38" customWidth="1" min="2" max="2"/>
-    <col width="14" customWidth="1" min="3" max="3"/>
+    <col width="16" customWidth="1" min="3" max="3"/>
     <col width="16" customWidth="1" min="4" max="4"/>
     <col width="12" customWidth="1" min="5" max="5"/>
+    <col width="24" customWidth="1" min="6" max="6"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -457,7 +458,7 @@
       </c>
       <c r="C1" s="1" t="inlineStr">
         <is>
-          <t>quarter</t>
+          <t>region</t>
         </is>
       </c>
       <c r="D1" s="1" t="inlineStr">
@@ -470,12 +471,17 @@
           <t>year</t>
         </is>
       </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
+          <t>delivery_type</t>
+        </is>
+      </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:E1000"/>
-  <dataValidations count="3">
+  <autoFilter ref="A1:F1000"/>
+  <dataValidations count="4">
     <dataValidation sqref="C2:C1000" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
-      <formula1>"Q1,Q2,Q3,Q4"</formula1>
+      <formula1>"ASIA,MENA,EUROPE,UK,LATAM,US"</formula1>
     </dataValidation>
     <dataValidation sqref="D2:D1000" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"January,February,March,April,May,June,July,August,September,October,November,December"</formula1>
@@ -483,6 +489,9 @@
     <dataValidation sqref="E2:E1000" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="whole" operator="between">
       <formula1>2020</formula1>
       <formula2>2100</formula2>
+    </dataValidation>
+    <dataValidation sqref="F2:F1000" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+      <formula1>"Feature,Run,New Market Deployment"</formula1>
     </dataValidation>
   </dataValidations>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -495,7 +504,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A7"/>
+  <dimension ref="A1:A9"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="95" customWidth="1" min="1" max="1"/>
@@ -518,28 +527,42 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>Required columns: application, feature_name, quarter, month, year.</t>
+          <t>Required columns: application, feature_name, region, month, year, delivery_type.</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>Use quarter values: Q1, Q2, Q3, Q4.</t>
+          <t>Quarter is auto-generated by the application based on month + year.</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>Use full month names (for example, January).</t>
+          <t>Region must be one of: ASIA, MENA, EUROPE, UK, LATAM, US.</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
+          <t>Use full month names (for example, January).</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
           <t>Use a 4-digit year (for example, 2026).</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>Delivery type must be one of: Feature, Run, New Market Deployment.</t>
         </is>
       </c>
     </row>

</xml_diff>